<commit_message>
Rename LCOS enclosure IDs so C# matches the radio address.
East End signals are C2 (radio 2) and turnouts C12 (radio 12); sequential C1–C13 labels stay in Legacy Node ID. Packed MQTT numbers are unchanged.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/cats/data/signals_asbuilt_abs_v2.xlsx
+++ b/cats/data/signals_asbuilt_abs_v2.xlsx
@@ -1280,7 +1280,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1290,7 +1290,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>C4-OU2-1 C4-OU2-3 C4-OU2-2</t>
+          <t>C3-OU2-1 C3-OU2-3 C3-OU2-2</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>C4-OU2-4 C4-OU2-6 C4-OU2-5</t>
+          <t>C3-OU2-4 C3-OU2-6 C3-OU2-5</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -1430,7 +1430,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1440,7 +1440,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>C4-OU3-4 C4-OU3-6 C4-OU3-5</t>
+          <t>C3-OU3-4 C3-OU3-6 C3-OU3-5</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1515,7 +1515,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>C4-OU3-7 C4-OU3-8 C4-OU2-7</t>
+          <t>C3-OU3-7 C3-OU3-8 C3-OU2-7</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1590,7 +1590,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>C4-OU3-1 C4-OU3-3 C4-OU3-2</t>
+          <t>C3-OU3-1 C3-OU3-3 C3-OU3-2</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>C13</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>C5-OU1-1 C5-OU1-3 C5-OU1-2</t>
+          <t>C13-OU1-1 C13-OU1-3 C13-OU1-2</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1730,7 +1730,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>C13</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>C5-OU1-4 C5-OU1-5 C5-OU1-6</t>
+          <t>C13-OU1-4 C13-OU1-5 C13-OU1-6</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1805,7 +1805,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>C13</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1815,7 +1815,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>C5-OU2-1 C5-OU2-3 C5-OU2-2</t>
+          <t>C13-OU2-1 C13-OU2-3 C13-OU2-2</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>C13</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>C5-OU2-4 C5-OU2-6 C5-OU2-5</t>
+          <t>C13-OU2-4 C13-OU2-6 C13-OU2-5</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1955,7 +1955,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>C3-OU1-1 C3-OU1-3 C3-OU1-2</t>
+          <t>C2-OU1-1 C2-OU1-3 C2-OU1-2</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was C3-OU1 new 5V</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was C2-OU1 5V (was C3)</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -2040,7 +2040,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>C3-OU1-4 C3-OU1-6 C3-OU1-5</t>
+          <t>C2-OU1-4 C2-OU1-6 C2-OU1-5</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was C3-OU1 new 5V</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was C2-OU1 5V (was C3)</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2105,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>C3-OU1-7 C3-OU2-1 C3-OU1-8</t>
+          <t>C2-OU1-7 C2-OU2-1 C2-OU1-8</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -2190,7 +2190,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>C3-OU2-2 C3-OU2-4 C3-OU2-3</t>
+          <t>C2-OU2-2 C2-OU2-4 C2-OU2-3</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -2255,7 +2255,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>C3-OU2-5 C3-OU2-7 C3-OU2-6</t>
+          <t>C2-OU2-5 C2-OU2-7 C2-OU2-6</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2330,7 +2330,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -2340,7 +2340,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>C3-OU3-1 C3-OU3-3 C3-OU3-2</t>
+          <t>C2-OU3-1 C2-OU3-3 C2-OU3-2</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -2780,7 +2780,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>C7</t>
+          <t>C11</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2790,7 +2790,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>C7-OU2-1 C7-OU2-2 C7-OU2-3</t>
+          <t>C11-OU2-1 C11-OU2-2 C11-OU2-3</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -2851,7 +2851,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>C7</t>
+          <t>C11</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2861,7 +2861,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>C7-OU2-4 C7-OU2-5 C7-OU2-6</t>
+          <t>C11-OU2-4 C11-OU2-5 C11-OU2-6</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>C7</t>
+          <t>C11</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2932,7 +2932,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>C7-OU3-1 C7-OU3-2 C7-OU3-3</t>
+          <t>C11-OU3-1 C11-OU3-2 C11-OU3-3</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">

</xml_diff>

<commit_message>
Add four 5V OU4 boards and wire both discs on every two-head mast.
Second lamps stay on the same radio as the top disc; C11 uses leftover OU3 instead of a new board. tables.xml is unchanged.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/cats/data/signals_asbuilt_abs_v2.xlsx
+++ b/cats/data/signals_asbuilt_abs_v2.xlsx
@@ -1256,7 +1256,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -1285,32 +1285,32 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>432</t>
+          <t>432 433</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>C3-OU2-1 C3-OU2-3 C3-OU2-2</t>
+          <t>C3-OU2-1 C3-OU2-3 C3-OU2-2 C3-OU4-1 C3-OU4-3 C3-OU4-2</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>track/signalhead/432</t>
+          <t>track/signalhead/432 track/signalhead/433</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH432)</t>
+          <t>IF$shsm:hart-aar:SL-2-digicon(IH432)(IH433)</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>AAR-1946 SL-1-low (3-pin STOP/APPROACH/CLEAR)</t>
+          <t>hart-aar SL-2-digicon (two 3-pin STOP/APPROACH/CLEAR discs)</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1556,7 +1556,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1585,32 +1585,32 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>438</t>
+          <t>438 439</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>C3-OU3-1 C3-OU3-3 C3-OU3-2</t>
+          <t>C3-OU3-1 C3-OU3-3 C3-OU3-2 C3-OU4-4 C3-OU4-6 C3-OU4-5</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>track/signalhead/438</t>
+          <t>track/signalhead/438 track/signalhead/439</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH438)</t>
+          <t>IF$shsm:hart-aar:SL-2-digicon(IH438)(IH439)</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>AAR-1946 SL-1-low (3-pin STOP/APPROACH/CLEAR)</t>
+          <t>hart-aar SL-2-digicon (two 3-pin STOP/APPROACH/CLEAR discs)</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1660,32 +1660,32 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>1332</t>
+          <t>1332 1333</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>C13-OU1-1 C13-OU1-3 C13-OU1-2</t>
+          <t>C13-OU1-1 C13-OU1-3 C13-OU1-2 C13-OU4-1 C13-OU4-3 C13-OU4-2</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>track/signalhead/1332</t>
+          <t>track/signalhead/1332 track/signalhead/1333</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH1332)</t>
+          <t>IF$shsm:hart-aar:SL-2-digicon(IH1332)(IH1333)</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>AAR-1946 SL-1-low (3-pin STOP/APPROACH/CLEAR)</t>
+          <t>hart-aar SL-2-digicon (two 3-pin STOP/APPROACH/CLEAR discs)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -1706,7 +1706,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1735,32 +1735,32 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>1335</t>
+          <t>1335 1336</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>C13-OU1-4 C13-OU1-5 C13-OU1-6</t>
+          <t>C13-OU1-4 C13-OU1-5 C13-OU1-6 C13-OU4-4 C13-OU4-6 C13-OU4-5</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>track/signalhead/1335</t>
+          <t>track/signalhead/1335 track/signalhead/1336</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH1335)</t>
+          <t>IF$shsm:hart-aar:SL-2-digicon(IH1335)(IH1336)</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>AAR-1946 SL-1-low (3-pin STOP/APPROACH/CLEAR)</t>
+          <t>hart-aar SL-2-digicon (two 3-pin STOP/APPROACH/CLEAR discs)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -1856,7 +1856,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1885,32 +1885,32 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>1337</t>
+          <t>1337 1338</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>C13-OU2-4 C13-OU2-6 C13-OU2-5</t>
+          <t>C13-OU2-4 C13-OU2-6 C13-OU2-5 C13-OU4-7 C13-OU2-8 C13-OU4-8</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>track/signalhead/1337</t>
+          <t>track/signalhead/1337 track/signalhead/1338</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH1337)</t>
+          <t>IF$shsm:hart-aar:SL-2-digicon(IH1337)(IH1338)</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>AAR-1946 SL-1-low (3-pin STOP/APPROACH/CLEAR)</t>
+          <t>hart-aar SL-2-digicon (two 3-pin STOP/APPROACH/CLEAR discs)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1931,7 +1931,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1960,37 +1960,37 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>232</t>
+          <t>232 238</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>C2-OU1-1 C2-OU1-3 C2-OU1-2</t>
+          <t>C2-OU1-1 C2-OU1-3 C2-OU1-2 C2-OU4-1 C2-OU4-3 C2-OU4-2</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>track/signalhead/232</t>
+          <t>track/signalhead/232 track/signalhead/238</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH232)</t>
+          <t>IF$shsm:hart-aar:SL-2-digicon(IH232)(IH238)</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>AAR-1946 SL-1-low (3-pin STOP/APPROACH/CLEAR)</t>
+          <t>hart-aar SL-2-digicon (two 3-pin STOP/APPROACH/CLEAR discs)</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was C2-OU1 5V (was C3)</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was C2-OU1 5V</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -2035,37 +2035,37 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>233 239</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>C2-OU1-4 C2-OU1-6 C2-OU1-5</t>
+          <t>C2-OU1-4 C2-OU1-6 C2-OU1-5 C2-OU4-4 C2-OU4-6 C2-OU4-5</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>track/signalhead/233</t>
+          <t>track/signalhead/233 track/signalhead/239</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH233)</t>
+          <t>IF$shsm:hart-aar:SL-2-digicon(IH233)(IH239)</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>AAR-1946 SL-1-low (3-pin STOP/APPROACH/CLEAR)</t>
+          <t>hart-aar SL-2-digicon (two 3-pin STOP/APPROACH/CLEAR discs)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was C2-OU1 5V (was C3)</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was C2-OU1 5V</t>
         </is>
       </c>
     </row>
@@ -2156,7 +2156,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -2185,32 +2185,32 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>235</t>
+          <t>235 240</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>C2-OU2-2 C2-OU2-4 C2-OU2-3</t>
+          <t>C2-OU2-2 C2-OU2-4 C2-OU2-3 C2-OU4-7 C2-OU3-7 C2-OU4-8</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>track/signalhead/235</t>
+          <t>track/signalhead/235 track/signalhead/240</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH235)</t>
+          <t>IF$shsm:hart-aar:SL-2-digicon(IH235)(IH240)</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>AAR-1946 SL-1-low (3-pin STOP/APPROACH/CLEAR)</t>
+          <t>hart-aar SL-2-digicon (two 3-pin STOP/APPROACH/CLEAR discs)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -2306,7 +2306,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -2335,32 +2335,32 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>237</t>
+          <t>237 241</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>C2-OU3-1 C2-OU3-3 C2-OU3-2</t>
+          <t>C2-OU3-1 C2-OU3-3 C2-OU3-2 C2-OU3-4 C2-OU3-6 C2-OU3-5</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>track/signalhead/237</t>
+          <t>track/signalhead/237 track/signalhead/241</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH237)</t>
+          <t>IF$shsm:hart-aar:SL-2-digicon(IH237)(IH241)</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>AAR-1946 SL-1-low (3-pin STOP/APPROACH/CLEAR)</t>
+          <t>hart-aar SL-2-digicon (two 3-pin STOP/APPROACH/CLEAR discs)</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -2381,7 +2381,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -2410,32 +2410,32 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>132 133</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>C1-OU2-1 C1-OU2-3 C1-OU2-2</t>
+          <t>C1-OU2-1 C1-OU2-3 C1-OU2-2 C1-OU4-1 C1-OU4-3 C1-OU4-2</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>track/signalhead/132</t>
+          <t>track/signalhead/132 track/signalhead/133</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH132)</t>
+          <t>IF$shsm:hart-aar:SL-2-digicon(IH132)(IH133)</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>AAR-1946 SL-1-low (3-pin STOP/APPROACH/CLEAR)</t>
+          <t>hart-aar SL-2-digicon (two 3-pin STOP/APPROACH/CLEAR discs)</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -2456,7 +2456,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -2485,32 +2485,32 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>135</t>
+          <t>135 136</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>C1-OU2-4 C1-OU2-6 C1-OU2-5</t>
+          <t>C1-OU2-4 C1-OU2-6 C1-OU2-5 C1-OU4-4 C1-OU4-6 C1-OU4-5</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>track/signalhead/135</t>
+          <t>track/signalhead/135 track/signalhead/136</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH135)</t>
+          <t>IF$shsm:hart-aar:SL-2-digicon(IH135)(IH136)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>AAR-1946 SL-1-low (3-pin STOP/APPROACH/CLEAR)</t>
+          <t>hart-aar SL-2-digicon (two 3-pin STOP/APPROACH/CLEAR discs)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -2531,7 +2531,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -2560,32 +2560,32 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>139</t>
+          <t>139 140</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>C1-OU3-1 C1-OU3-3 C1-OU3-2</t>
+          <t>C1-OU3-1 C1-OU3-3 C1-OU3-2 C1-OU4-7 C1-OU2-8 C1-OU4-8</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>track/signalhead/139</t>
+          <t>track/signalhead/139 track/signalhead/140</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH139)</t>
+          <t>IF$shsm:hart-aar:SL-2-digicon(IH139)(IH140)</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>AAR-1946 SL-1-low (3-pin STOP/APPROACH/CLEAR)</t>
+          <t>hart-aar SL-2-digicon (two 3-pin STOP/APPROACH/CLEAR discs)</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -2756,7 +2756,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2785,32 +2785,32 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>1132</t>
+          <t>1132 1135</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>C11-OU2-1 C11-OU2-2 C11-OU2-3</t>
+          <t>C11-OU2-1 C11-OU2-2 C11-OU2-3 C11-OU3-4 C11-OU3-6 C11-OU3-5</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>track/signalhead/1132</t>
+          <t>track/signalhead/1132 track/signalhead/1135</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH1132)</t>
+          <t>IF$shsm:hart-aar:SL-2-digicon(IH1132)(IH1135)</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>AAR-1946 SL-1-low (3-pin STOP/APPROACH/CLEAR)</t>
+          <t>hart-aar SL-2-digicon (two 3-pin STOP/APPROACH/CLEAR discs)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">

</xml_diff>

<commit_message>
Group each two-head mast onto one DNOU8 so those boards can sit next to their plants.
A neighboring dwarf uses the leftover pins; the ninth lamp spills to the adjacent cluster. Packed MQTT IDs are unchanged.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/cats/data/signals_asbuilt_abs_v2.xlsx
+++ b/cats/data/signals_asbuilt_abs_v2.xlsx
@@ -1290,7 +1290,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>C3-OU2-1 C3-OU2-3 C3-OU2-2 C3-OU4-1 C3-OU4-3 C3-OU4-2</t>
+          <t>C3-OU2-1 C3-OU2-3 C3-OU2-2 C3-OU2-4 C3-OU2-6 C3-OU2-5</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>C3-OU2-4 C3-OU2-6 C3-OU2-5</t>
+          <t>C3-OU2-7 C3-OU3-7 C3-OU2-8</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -1390,7 +1390,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was S3-7 G/Y/R</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was G/Y on Plane OU2; R spills to 2L OU3</t>
         </is>
       </c>
     </row>
@@ -1402,25 +1402,25 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mast 4RA</t>
+          <t>Mast 2L</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>(4,3) LEFT</t>
+          <t>(8,3) RIGHT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Switch 3</t>
+          <t>Switch 1</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1435,37 +1435,37 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>436</t>
+          <t>438 439</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>C3-OU3-4 C3-OU3-6 C3-OU3-5</t>
+          <t>C3-OU3-1 C3-OU3-3 C3-OU3-2 C3-OU3-4 C3-OU3-6 C3-OU3-5</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>track/signalhead/436</t>
+          <t>track/signalhead/438 track/signalhead/439</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH436)</t>
+          <t>IF$shsm:hart-aar:SL-2-digicon(IH438)(IH439)</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>AAR-1946 SL-1-low (3-pin STOP/APPROACH/CLEAR)</t>
+          <t>hart-aar SL-2-digicon (two 3-pin STOP/APPROACH/CLEAR discs)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was S3-9 G/Y/R</t>
+          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp G; was S3-8 G/Y/R</t>
         </is>
       </c>
     </row>
@@ -1477,7 +1477,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Mast 4RB</t>
+          <t>Mast 4RA</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>(4,4) LEFT</t>
+          <t>(4,3) LEFT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1510,22 +1510,22 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>437</t>
+          <t>436</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>C3-OU3-7 C3-OU3-8 C3-OU2-7</t>
+          <t>C3-OU4-1 C3-OU4-3 C3-OU4-2</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>track/signalhead/437</t>
+          <t>track/signalhead/436</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH437)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH436)</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp G; was S3-11 G/Y/R (Y on OU2-7)</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was Brick west OU4 with 4RB</t>
         </is>
       </c>
     </row>
@@ -1552,25 +1552,25 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Mast 2L</t>
+          <t>Mast 4RB</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>(8,3) RIGHT</t>
+          <t>(4,4) LEFT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Switch 1</t>
+          <t>Switch 3</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1585,37 +1585,37 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>438 439</t>
+          <t>437</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>C3-OU3-1 C3-OU3-3 C3-OU3-2 C3-OU4-4 C3-OU4-6 C3-OU4-5</t>
+          <t>C3-OU4-4 C3-OU4-6 C3-OU4-5</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>track/signalhead/438 track/signalhead/439</t>
+          <t>track/signalhead/437</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH438)(IH439)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH437)</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>double</t>
+          <t>single</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>hart-aar SL-2-digicon (two 3-pin STOP/APPROACH/CLEAR discs)</t>
+          <t>AAR-1946 SL-1-low (3-pin STOP/APPROACH/CLEAR)</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp G; was S3-8 G/Y/R</t>
+          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp G; was Brick west OU4 with 4RA</t>
         </is>
       </c>
     </row>
@@ -1665,7 +1665,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>C13-OU1-1 C13-OU1-3 C13-OU1-2 C13-OU4-1 C13-OU4-3 C13-OU4-2</t>
+          <t>C13-OU1-1 C13-OU1-3 C13-OU1-2 C13-OU1-4 C13-OU1-6 C13-OU1-5</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>C13-OU1-4 C13-OU1-5 C13-OU1-6 C13-OU4-4 C13-OU4-6 C13-OU4-5</t>
+          <t>C13-OU4-1 C13-OU4-3 C13-OU4-2 C13-OU4-4 C13-OU4-6 C13-OU4-5</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1765,7 +1765,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp G; was S3-12 G/R/Y silk</t>
+          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp G; was S3-12; sequential G/Y/R</t>
         </is>
       </c>
     </row>
@@ -1777,11 +1777,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Mast 8LB</t>
+          <t>Mast 8LA</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>(14,7) RIGHT</t>
+          <t>(14,8) RIGHT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1810,37 +1810,37 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>1334</t>
+          <t>1337 1338</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>C13-OU2-1 C13-OU2-3 C13-OU2-2</t>
+          <t>C13-OU2-1 C13-OU2-3 C13-OU2-2 C13-OU2-4 C13-OU2-6 C13-OU2-5</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>track/signalhead/1334</t>
+          <t>track/signalhead/1337 track/signalhead/1338</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH1334)</t>
+          <t>IF$shsm:hart-aar:SL-2-digicon(IH1337)(IH1338)</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>AAR-1946 SL-1-low (3-pin STOP/APPROACH/CLEAR)</t>
+          <t>hart-aar SL-2-digicon (two 3-pin STOP/APPROACH/CLEAR discs)</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was S3-4 G/Y/R</t>
+          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp G; was S3-5 G/Y/R</t>
         </is>
       </c>
     </row>
@@ -1852,11 +1852,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Mast 8LA</t>
+          <t>Mast 8LB</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1865,7 +1865,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>(14,8) RIGHT</t>
+          <t>(14,7) RIGHT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1885,37 +1885,37 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>1337 1338</t>
+          <t>1334</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>C13-OU2-4 C13-OU2-6 C13-OU2-5 C13-OU4-7 C13-OU2-8 C13-OU4-8</t>
+          <t>C13-OU2-7 C13-OU4-7 C13-OU2-8</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>track/signalhead/1337 track/signalhead/1338</t>
+          <t>track/signalhead/1334</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH1337)(IH1338)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH1334)</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>double</t>
+          <t>single</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>hart-aar SL-2-digicon (two 3-pin STOP/APPROACH/CLEAR discs)</t>
+          <t>AAR-1946 SL-1-low (3-pin STOP/APPROACH/CLEAR)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp G; was S3-5 G/Y/R</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was G/Y with 8LA; R spills to 8RB OU4</t>
         </is>
       </c>
     </row>
@@ -1965,7 +1965,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>C2-OU1-1 C2-OU1-3 C2-OU1-2 C2-OU4-1 C2-OU4-3 C2-OU4-2</t>
+          <t>C2-OU1-1 C2-OU1-3 C2-OU1-2 C2-OU1-4 C2-OU1-6 C2-OU1-5</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -2002,20 +2002,20 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Mast 24L</t>
+          <t>Mast 24RB</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>(30,6) RIGHT</t>
+          <t>(28,7) LEFT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -2035,37 +2035,37 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>233 239</t>
+          <t>234</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>C2-OU1-4 C2-OU1-6 C2-OU1-5 C2-OU4-4 C2-OU4-6 C2-OU4-5</t>
+          <t>C2-OU1-7 C2-OU2-7 C2-OU1-8</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>track/signalhead/233 track/signalhead/239</t>
+          <t>track/signalhead/234</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH233)(IH239)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH234)</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>double</t>
+          <t>single</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>hart-aar SL-2-digicon (two 3-pin STOP/APPROACH/CLEAR discs)</t>
+          <t>AAR-1946 SL-1-low (3-pin STOP/APPROACH/CLEAR)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was C2-OU1 5V</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was G/Y with 24RA; R spills to 24L OU2</t>
         </is>
       </c>
     </row>
@@ -2077,20 +2077,20 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Mast 24RB</t>
+          <t>Mast 24L</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>(28,7) LEFT</t>
+          <t>(30,6) RIGHT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -2110,37 +2110,37 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>234</t>
+          <t>233 239</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>C2-OU1-7 C2-OU2-1 C2-OU1-8</t>
+          <t>C2-OU2-1 C2-OU2-3 C2-OU2-2 C2-OU2-4 C2-OU2-6 C2-OU2-5</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>track/signalhead/234</t>
+          <t>track/signalhead/233 track/signalhead/239</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH234)</t>
+          <t>IF$shsm:hart-aar:SL-2-digicon(IH233)(IH239)</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>AAR-1946 SL-1-low (3-pin STOP/APPROACH/CLEAR)</t>
+          <t>hart-aar SL-2-digicon (two 3-pin STOP/APPROACH/CLEAR discs)</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was OU1-7/8 + OU2-1</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was moved from OU1 with 24RA</t>
         </is>
       </c>
     </row>
@@ -2190,7 +2190,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>C2-OU2-2 C2-OU2-4 C2-OU2-3 C2-OU4-7 C2-OU3-7 C2-OU4-8</t>
+          <t>C2-OU3-1 C2-OU3-3 C2-OU3-2 C2-OU3-4 C2-OU3-6 C2-OU3-5</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>C2-OU2-5 C2-OU2-7 C2-OU2-6</t>
+          <t>C2-OU3-7 C2-OU4-7 C2-OU3-8</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2290,7 +2290,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was OU2-8 is relay</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was G/Y with 34L; R spills to 34R OU4</t>
         </is>
       </c>
     </row>
@@ -2340,7 +2340,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>C2-OU3-1 C2-OU3-3 C2-OU3-2 C2-OU3-4 C2-OU3-6 C2-OU3-5</t>
+          <t>C2-OU4-1 C2-OU4-3 C2-OU4-2 C2-OU4-4 C2-OU4-6 C2-OU4-5</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Mast 40LB</t>
+          <t>Mast 36RA</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2385,17 +2385,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>(43,5) RIGHT</t>
+          <t>(37,6) LEFT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Switch 39</t>
+          <t>Switch 35</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2410,22 +2410,22 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>132 133</t>
+          <t>135 136</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>C1-OU2-1 C1-OU2-3 C1-OU2-2 C1-OU4-1 C1-OU4-3 C1-OU4-2</t>
+          <t>C1-OU2-1 C1-OU2-3 C1-OU2-2 C1-OU2-4 C1-OU2-6 C1-OU2-5</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>track/signalhead/132 track/signalhead/133</t>
+          <t>track/signalhead/135 track/signalhead/136</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH132)(IH133)</t>
+          <t>IF$shsm:hart-aar:SL-2-digicon(IH135)(IH136)</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2440,7 +2440,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was S1-1 G/Y/R</t>
+          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp G; was S1-2 G/Y/R</t>
         </is>
       </c>
     </row>
@@ -2452,11 +2452,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Mast 36RA</t>
+          <t>Mast 40LA</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -2465,12 +2465,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>(37,6) LEFT</t>
+          <t>(43,6) RIGHT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Switch 35</t>
+          <t>Switch 39</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2485,37 +2485,37 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>135 136</t>
+          <t>142</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>C1-OU2-4 C1-OU2-6 C1-OU2-5 C1-OU4-4 C1-OU4-6 C1-OU4-5</t>
+          <t>C1-OU3-7 C1-OU2-7 C1-OU3-8</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>track/signalhead/135 track/signalhead/136</t>
+          <t>track/signalhead/142</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH135)(IH136)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH142)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>double</t>
+          <t>single</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>hart-aar SL-2-digicon (two 3-pin STOP/APPROACH/CLEAR discs)</t>
+          <t>AAR-1946 SL-1-low (3-pin STOP/APPROACH/CLEAR)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp G; was S1-2 G/Y/R</t>
+          <t>LCOS Signal 10 UID 42; STOP/APPROACH/CLEAR; lamp G; was G/Y with 40LB; R spills to 36RA OU2</t>
         </is>
       </c>
     </row>
@@ -2527,7 +2527,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Mast 38LB</t>
+          <t>Mast 40LB</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2540,12 +2540,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>(43,8) RIGHT</t>
+          <t>(43,5) RIGHT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Switch 37</t>
+          <t>Switch 39</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2560,22 +2560,22 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>139 140</t>
+          <t>132 133</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>C1-OU3-1 C1-OU3-3 C1-OU3-2 C1-OU4-7 C1-OU2-8 C1-OU4-8</t>
+          <t>C1-OU3-1 C1-OU3-3 C1-OU3-2 C1-OU3-4 C1-OU3-6 C1-OU3-5</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>track/signalhead/139 track/signalhead/140</t>
+          <t>track/signalhead/132 track/signalhead/133</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH139)(IH140)</t>
+          <t>IF$shsm:hart-aar:SL-2-digicon(IH132)(IH133)</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2590,7 +2590,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp G; was S1-3 G/Y/R</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was S1-1 G/Y/R</t>
         </is>
       </c>
     </row>
@@ -2602,7 +2602,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Mast 40LA</t>
+          <t>Mast 38LA</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2615,12 +2615,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>(43,6) RIGHT</t>
+          <t>(43,7) RIGHT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Switch 39</t>
+          <t>Switch 37</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2635,22 +2635,22 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>143</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>C1-OU3-4 C1-OU3-6 C1-OU3-5</t>
+          <t>C1-OU4-7 C1-OU2-8 C1-OU4-8</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>track/signalhead/142</t>
+          <t>track/signalhead/143</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH142)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH143)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>LCOS Signal 10 UID 42; STOP/APPROACH/CLEAR; lamp G; was S1-4 G/Y/R</t>
+          <t>LCOS Signal 11 UID 43; STOP/APPROACH/CLEAR; lamp G; was G/Y with 38LB; R spills to 36RA OU2</t>
         </is>
       </c>
     </row>
@@ -2677,20 +2677,20 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Mast 38LA</t>
+          <t>Mast 38LB</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>(43,7) RIGHT</t>
+          <t>(43,8) RIGHT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2710,37 +2710,37 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>143</t>
+          <t>139 140</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>C1-OU2-7 C1-OU3-8 C1-OU3-7</t>
+          <t>C1-OU4-1 C1-OU4-3 C1-OU4-2 C1-OU4-4 C1-OU4-6 C1-OU4-5</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>track/signalhead/143</t>
+          <t>track/signalhead/139 track/signalhead/140</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH143)</t>
+          <t>IF$shsm:hart-aar:SL-2-digicon(IH139)(IH140)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>AAR-1946 SL-1-low (3-pin STOP/APPROACH/CLEAR)</t>
+          <t>hart-aar SL-2-digicon (two 3-pin STOP/APPROACH/CLEAR discs)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>LCOS Signal 11 UID 43; STOP/APPROACH/CLEAR; lamp G; was spares G/Y/R</t>
+          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp G; was S1-3 G/Y/R</t>
         </is>
       </c>
     </row>
@@ -2790,7 +2790,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>C11-OU2-1 C11-OU2-2 C11-OU2-3 C11-OU3-4 C11-OU3-6 C11-OU3-5</t>
+          <t>C11-OU2-1 C11-OU2-3 C11-OU2-2 C11-OU2-4 C11-OU2-6 C11-OU2-5</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -2815,7 +2815,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was S1-5 G/R/Y silk</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was S1-5; sequential G/Y/R</t>
         </is>
       </c>
     </row>
@@ -2861,7 +2861,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>C11-OU2-4 C11-OU2-5 C11-OU2-6</t>
+          <t>C11-OU3-1 C11-OU3-3 C11-OU3-2</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was S1-6 G/R/Y silk</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was S1-6; sequential G/Y/R</t>
         </is>
       </c>
     </row>
@@ -2932,7 +2932,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>C11-OU3-1 C11-OU3-2 C11-OU3-3</t>
+          <t>C11-OU3-4 C11-OU3-6 C11-OU3-5</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2957,7 +2957,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was S4-6 G/R/Y silk</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was S4-6; sequential G/Y/R</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Put Digicon heads on the cabinet already at each plant.
C4 takes Brick+Plane, C12 takes East End 34, C2 keeps only the west 24 overflow, C11 takes Princess 40 plus the balloon, and C3 no longer carries signal pins.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/cats/data/signals_asbuilt_abs_v2.xlsx
+++ b/cats/data/signals_asbuilt_abs_v2.xlsx
@@ -1280,7 +1280,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1290,7 +1290,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>C3-OU2-1 C3-OU2-3 C3-OU2-2 C3-OU2-4 C3-OU2-6 C3-OU2-5</t>
+          <t>C4-OU2-1 C4-OU2-3 C4-OU2-2 C4-OU2-4 C4-OU2-6 C4-OU2-5</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>C3-OU2-7 C3-OU3-7 C3-OU2-8</t>
+          <t>C4-OU2-7 C4-OU3-7 C4-OU2-8</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -1430,7 +1430,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1440,7 +1440,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>C3-OU3-1 C3-OU3-3 C3-OU3-2 C3-OU3-4 C3-OU3-6 C3-OU3-5</t>
+          <t>C4-OU3-1 C4-OU3-3 C4-OU3-2 C4-OU3-4 C4-OU3-6 C4-OU3-5</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1515,7 +1515,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>C3-OU4-1 C3-OU4-3 C3-OU4-2</t>
+          <t>C4-OU4-1 C4-OU4-3 C4-OU4-2</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1590,7 +1590,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>C3-OU4-4 C3-OU4-6 C3-OU4-5</t>
+          <t>C4-OU4-4 C4-OU4-6 C4-OU4-5</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was moved from OU1 with 24RA</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was with 24RA cluster</t>
         </is>
       </c>
     </row>
@@ -2175,32 +2175,32 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C12</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>235 240</t>
+          <t>1232 1233</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>C2-OU3-1 C2-OU3-3 C2-OU3-2 C2-OU3-4 C2-OU3-6 C2-OU3-5</t>
+          <t>C12-OU2-1 C12-OU2-3 C12-OU2-2 C12-OU2-4 C12-OU2-6 C12-OU2-5</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>track/signalhead/235 track/signalhead/240</t>
+          <t>track/signalhead/1232 track/signalhead/1233</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH235)(IH240)</t>
+          <t>IF$shsm:hart-aar:SL-2-digicon(IH1232)(IH1233)</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -2215,7 +2215,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp G; was was S2-5/S2-3 mix</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was was C2 235</t>
         </is>
       </c>
     </row>
@@ -2250,32 +2250,32 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C12</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>1234</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>C2-OU3-7 C2-OU4-7 C2-OU3-8</t>
+          <t>C12-OU2-7 C12-OU3-7 C12-OU2-8</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>track/signalhead/236</t>
+          <t>track/signalhead/1234</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH236)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH1234)</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2290,7 +2290,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was G/Y with 34L; R spills to 34R OU4</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was G/Y with 34L; R spills to 34R OU3</t>
         </is>
       </c>
     </row>
@@ -2325,32 +2325,32 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C12</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>237 241</t>
+          <t>1235 1236</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>C2-OU4-1 C2-OU4-3 C2-OU4-2 C2-OU4-4 C2-OU4-6 C2-OU4-5</t>
+          <t>C12-OU3-1 C12-OU3-3 C12-OU3-2 C12-OU3-4 C12-OU3-6 C12-OU3-5</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>track/signalhead/237 track/signalhead/241</t>
+          <t>track/signalhead/1235 track/signalhead/1236</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH237)(IH241)</t>
+          <t>IF$shsm:hart-aar:SL-2-digicon(IH1235)(IH1236)</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2365,7 +2365,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp G; was was S4-6 G/R/Y</t>
+          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp G; was was C2 237</t>
         </is>
       </c>
     </row>
@@ -2452,11 +2452,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Mast 40LA</t>
+          <t>Mast 36RB</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -2465,12 +2465,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>(43,6) RIGHT</t>
+          <t>(37,7) LEFT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Switch 39</t>
+          <t>Switch 35</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2485,37 +2485,37 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>132 133</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>C1-OU3-7 C1-OU2-7 C1-OU3-8</t>
+          <t>C1-OU3-1 C1-OU3-3 C1-OU3-2 C1-OU3-4 C1-OU3-6 C1-OU3-5</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>track/signalhead/142</t>
+          <t>track/signalhead/132 track/signalhead/133</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH142)</t>
+          <t>IF$shsm:hart-aar:SL-2-digicon(IH132)(IH133)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>AAR-1946 SL-1-low (3-pin STOP/APPROACH/CLEAR)</t>
+          <t>hart-aar SL-2-digicon (two 3-pin STOP/APPROACH/CLEAR discs)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>LCOS Signal 10 UID 42; STOP/APPROACH/CLEAR; lamp G; was G/Y with 40LB; R spills to 36RA OU2</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was was C11 1132</t>
         </is>
       </c>
     </row>
@@ -2527,7 +2527,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Mast 40LB</t>
+          <t>Mast 38LB</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2540,12 +2540,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>(43,5) RIGHT</t>
+          <t>(43,8) RIGHT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Switch 39</t>
+          <t>Switch 37</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2560,22 +2560,22 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>132 133</t>
+          <t>139 140</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>C1-OU3-1 C1-OU3-3 C1-OU3-2 C1-OU3-4 C1-OU3-6 C1-OU3-5</t>
+          <t>C1-OU4-1 C1-OU4-3 C1-OU4-2 C1-OU4-4 C1-OU4-6 C1-OU4-5</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>track/signalhead/132 track/signalhead/133</t>
+          <t>track/signalhead/139 track/signalhead/140</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH132)(IH133)</t>
+          <t>IF$shsm:hart-aar:SL-2-digicon(IH139)(IH140)</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2590,7 +2590,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was S1-1 G/Y/R</t>
+          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp G; was S1-3 G/Y/R</t>
         </is>
       </c>
     </row>
@@ -2640,7 +2640,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>C1-OU4-7 C1-OU2-8 C1-OU4-8</t>
+          <t>C1-OU4-7 C1-OU2-7 C1-OU4-8</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -2677,7 +2677,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Mast 38LB</t>
+          <t>Mast 40LB</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2690,42 +2690,42 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>(43,8) RIGHT</t>
+          <t>(43,5) RIGHT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Switch 37</t>
+          <t>Switch 39</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>C11</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>139 140</t>
+          <t>1132 1135</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>C1-OU4-1 C1-OU4-3 C1-OU4-2 C1-OU4-4 C1-OU4-6 C1-OU4-5</t>
+          <t>C11-OU2-1 C11-OU2-3 C11-OU2-2 C11-OU2-4 C11-OU2-6 C11-OU2-5</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>track/signalhead/139 track/signalhead/140</t>
+          <t>track/signalhead/1132 track/signalhead/1135</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH139)(IH140)</t>
+          <t>IF$shsm:hart-aar:SL-2-digicon(IH1132)(IH1135)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2740,7 +2740,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp G; was S1-3 G/Y/R</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was was C1 132</t>
         </is>
       </c>
     </row>
@@ -2752,11 +2752,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Mast 36RB</t>
+          <t>Mast 40LA</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2765,12 +2765,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>(37,7) LEFT</t>
+          <t>(43,6) RIGHT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Switch 35</t>
+          <t>Switch 39</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2785,37 +2785,37 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>1132 1135</t>
+          <t>1136</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>C11-OU2-1 C11-OU2-3 C11-OU2-2 C11-OU2-4 C11-OU2-6 C11-OU2-5</t>
+          <t>C11-OU2-7 C11-OU3-7 C11-OU2-8</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>track/signalhead/1132 track/signalhead/1135</t>
+          <t>track/signalhead/1136</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH1132)(IH1135)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH1136)</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>double</t>
+          <t>single</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>hart-aar SL-2-digicon (two 3-pin STOP/APPROACH/CLEAR discs)</t>
+          <t>AAR-1946 SL-1-low (3-pin STOP/APPROACH/CLEAR)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was S1-5; sequential G/Y/R</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was G/Y with 40LB; R spills to balloon OU3</t>
         </is>
       </c>
     </row>

</xml_diff>